<commit_message>
self test module skeleton and optimization
</commit_message>
<xml_diff>
--- a/assets/Releases/Release_plan.xlsx
+++ b/assets/Releases/Release_plan.xlsx
@@ -5,16 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\friday\rtos_pico\feb2\Robo_dev\assets\Releases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\home\friday\rtos_pico\feb2\Robo_dev\assets\Releases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{789704D9-888E-46CC-A6CC-0DECC02DAA35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDD7B1A-B674-4D9E-80C6-CC6308388CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-4815" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Analysis" sheetId="1" r:id="rId1"/>
+    <sheet name="Revision Histoy" sheetId="1" r:id="rId1"/>
     <sheet name="Release" sheetId="2" r:id="rId2"/>
+    <sheet name="HLD" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="73">
   <si>
     <t>S.No.</t>
   </si>
@@ -122,13 +123,136 @@
   </si>
   <si>
     <t>SW100</t>
+  </si>
+  <si>
+    <t>Authur</t>
+  </si>
+  <si>
+    <t>ASW1</t>
+  </si>
+  <si>
+    <t>ASW2</t>
+  </si>
+  <si>
+    <t>ASW3</t>
+  </si>
+  <si>
+    <t>ASW4</t>
+  </si>
+  <si>
+    <t>ASW5</t>
+  </si>
+  <si>
+    <t>ASW6</t>
+  </si>
+  <si>
+    <t>*ASW</t>
+  </si>
+  <si>
+    <t>Application Software</t>
+  </si>
+  <si>
+    <t>*RTE</t>
+  </si>
+  <si>
+    <t>Runtime Environment</t>
+  </si>
+  <si>
+    <t>RTE</t>
+  </si>
+  <si>
+    <t>BSW1</t>
+  </si>
+  <si>
+    <t>BSW2</t>
+  </si>
+  <si>
+    <t>BSW3</t>
+  </si>
+  <si>
+    <t>*BSW</t>
+  </si>
+  <si>
+    <t>Basic Software</t>
+  </si>
+  <si>
+    <t>OS</t>
+  </si>
+  <si>
+    <t>(freeRtos)</t>
+  </si>
+  <si>
+    <t>CDD</t>
+  </si>
+  <si>
+    <t>SYS1</t>
+  </si>
+  <si>
+    <t>SYS2</t>
+  </si>
+  <si>
+    <t>SYS3</t>
+  </si>
+  <si>
+    <t>Mcal1</t>
+  </si>
+  <si>
+    <t>Mcal2</t>
+  </si>
+  <si>
+    <t>Mcal3</t>
+  </si>
+  <si>
+    <t>Mcal4</t>
+  </si>
+  <si>
+    <t>*SYS</t>
+  </si>
+  <si>
+    <t>System Software</t>
+  </si>
+  <si>
+    <t>Pico-SDK</t>
+  </si>
+  <si>
+    <t>High-Level Design</t>
+  </si>
+  <si>
+    <t>*CDD</t>
+  </si>
+  <si>
+    <t>Complex Device driver</t>
+  </si>
+  <si>
+    <t>*MCAL</t>
+  </si>
+  <si>
+    <t>MicroController abstraction layer</t>
+  </si>
+  <si>
+    <t>blink</t>
+  </si>
+  <si>
+    <t>Nvm</t>
+  </si>
+  <si>
+    <t>Servo</t>
+  </si>
+  <si>
+    <t>Tools</t>
+  </si>
+  <si>
+    <t>*Tools</t>
+  </si>
+  <si>
+    <t>gpt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -150,16 +274,82 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF99FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF5050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCCFF33"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF99FFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -167,28 +357,200 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF405DEC"/>
+      <color rgb="FFFF5050"/>
+      <color rgb="FF99FFCC"/>
+      <color rgb="FFCC66FF"/>
+      <color rgb="FF9966FF"/>
+      <color rgb="FFCCFF33"/>
+      <color rgb="FFFF99FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -472,46 +834,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{835A3CD6-3E76-41D7-87C5-598825025B98}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.42578125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.42578125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="2">
         <v>46020</v>
       </c>
       <c r="E2" t="s">
@@ -520,28 +886,31 @@
       <c r="F2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B3" s="2" t="s">
+      <c r="G2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="2">
         <v>46021</v>
       </c>
       <c r="E5" t="s">
@@ -550,18 +919,21 @@
       <c r="F5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="2">
         <v>46021</v>
       </c>
       <c r="E6" t="s">
@@ -570,18 +942,21 @@
       <c r="F6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>4</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="2">
         <v>46021</v>
       </c>
       <c r="E7" t="s">
@@ -590,23 +965,26 @@
       <c r="F7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
+      <c r="G7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>5</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="2">
         <v>46021</v>
       </c>
       <c r="E9" t="s">
@@ -615,18 +993,21 @@
       <c r="F9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="G9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="2">
         <v>46022</v>
       </c>
       <c r="E10" t="s">
@@ -635,18 +1016,21 @@
       <c r="F10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="G10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>7</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="2">
         <v>46022</v>
       </c>
       <c r="E11" t="s">
@@ -655,18 +1039,21 @@
       <c r="F11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="G11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>8</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="2">
         <v>46022</v>
       </c>
       <c r="E12" t="s">
@@ -675,18 +1062,21 @@
       <c r="F12" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="G12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>9</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="2">
         <v>46022</v>
       </c>
       <c r="E13" t="s">
@@ -695,28 +1085,374 @@
       <c r="F13" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="G13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>10</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="2">
         <v>46054</v>
       </c>
       <c r="E14" t="s">
         <v>6</v>
       </c>
       <c r="F14" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C101226D-F072-4A6B-9A78-5314D6A47802}">
+  <dimension ref="A2:X22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="10.140625" customWidth="1"/>
+    <col min="24" max="24" width="30.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F5" s="62"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="59" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" s="8"/>
+      <c r="J5" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" s="8"/>
+      <c r="L5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="M5" s="8"/>
+      <c r="N5" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O5" s="8"/>
+      <c r="P5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="S5" s="8"/>
+      <c r="W5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="X5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F6" s="64" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" s="65"/>
+      <c r="H6" s="60"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="10"/>
+      <c r="W6" s="55" t="s">
+        <v>41</v>
+      </c>
+      <c r="X6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F7" s="64"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M7" s="11"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
+      <c r="R7" s="28"/>
+      <c r="S7" s="29"/>
+      <c r="W7" s="56" t="s">
+        <v>47</v>
+      </c>
+      <c r="X7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F8" s="64"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="43"/>
+      <c r="L8" s="30"/>
+      <c r="M8" s="30"/>
+      <c r="N8" s="30"/>
+      <c r="O8" s="30"/>
+      <c r="P8" s="43"/>
+      <c r="Q8" s="43"/>
+      <c r="R8" s="30"/>
+      <c r="S8" s="31"/>
+      <c r="W8" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="X8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F9" s="64"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="I9" s="49"/>
+      <c r="J9" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="K9" s="13"/>
+      <c r="L9" s="37" t="s">
+        <v>45</v>
+      </c>
+      <c r="M9" s="27"/>
+      <c r="N9" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="O9" s="37"/>
+      <c r="P9" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="41" t="s">
+        <v>51</v>
+      </c>
+      <c r="S9" s="32"/>
+      <c r="W9" s="57" t="s">
+        <v>63</v>
+      </c>
+      <c r="X9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F10" s="64"/>
+      <c r="G10" s="65"/>
+      <c r="H10" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="I10" s="49"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="27"/>
+      <c r="L10" s="38"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="38"/>
+      <c r="P10" s="47"/>
+      <c r="Q10" s="48"/>
+      <c r="R10" s="42"/>
+      <c r="S10" s="34"/>
+      <c r="W10" s="58" t="s">
+        <v>65</v>
+      </c>
+      <c r="X10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F11" s="64"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="49"/>
+      <c r="I11" s="49"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="39" t="s">
+        <v>52</v>
+      </c>
+      <c r="M11" s="17"/>
+      <c r="N11" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="O11" s="39"/>
+      <c r="P11" s="47"/>
+      <c r="Q11" s="48"/>
+      <c r="R11" s="42"/>
+      <c r="S11" s="34"/>
+    </row>
+    <row r="12" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F12" s="64"/>
+      <c r="G12" s="65"/>
+      <c r="H12" s="49"/>
+      <c r="I12" s="49"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="40"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="40"/>
+      <c r="P12" s="18"/>
+      <c r="Q12" s="19"/>
+      <c r="R12" s="42"/>
+      <c r="S12" s="34"/>
+    </row>
+    <row r="13" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F13" s="64"/>
+      <c r="G13" s="65"/>
+      <c r="H13" s="49"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="44" t="s">
+        <v>55</v>
+      </c>
+      <c r="K13" s="45"/>
+      <c r="L13" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="M13" s="21"/>
+      <c r="N13" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="O13" s="21"/>
+      <c r="P13" s="44" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q13" s="45"/>
+      <c r="R13" s="33"/>
+      <c r="S13" s="34"/>
+    </row>
+    <row r="14" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F14" s="64"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="22"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="22"/>
+      <c r="M14" s="23"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="23"/>
+      <c r="P14" s="22"/>
+      <c r="Q14" s="23"/>
+      <c r="R14" s="35"/>
+      <c r="S14" s="36"/>
+    </row>
+    <row r="15" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F15" s="64"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="50"/>
+      <c r="J15" s="50"/>
+      <c r="K15" s="50"/>
+      <c r="L15" s="54" t="s">
+        <v>61</v>
+      </c>
+      <c r="M15" s="54"/>
+      <c r="N15" s="50"/>
+      <c r="O15" s="50"/>
+      <c r="P15" s="50"/>
+      <c r="Q15" s="50"/>
+      <c r="R15" s="50"/>
+      <c r="S15" s="51"/>
+    </row>
+    <row r="16" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F16" s="66"/>
+      <c r="G16" s="67"/>
+      <c r="H16" s="52"/>
+      <c r="I16" s="52"/>
+      <c r="J16" s="52"/>
+      <c r="K16" s="52"/>
+      <c r="L16" s="52"/>
+      <c r="M16" s="52"/>
+      <c r="N16" s="52"/>
+      <c r="O16" s="52"/>
+      <c r="P16" s="52"/>
+      <c r="Q16" s="52"/>
+      <c r="R16" s="52"/>
+      <c r="S16" s="53"/>
+    </row>
+    <row r="18" spans="1:10" s="68" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B20" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="F20" s="57" t="s">
+        <v>63</v>
+      </c>
+      <c r="H20" s="64" t="s">
+        <v>71</v>
+      </c>
+      <c r="J20" s="58" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>1</v>
+      </c>
+      <c r="B22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22" t="s">
+        <v>69</v>
+      </c>
+      <c r="I22">
+        <v>1</v>
+      </c>
+      <c r="J22" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="L15:M15"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
swd debug scripts added
</commit_message>
<xml_diff>
--- a/assets/Releases/Release_plan.xlsx
+++ b/assets/Releases/Release_plan.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\friday\rtos_pico\feb2\Robo_dev\assets\Releases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\friday\rtos_pico\may17\Robo_dev\assets\Releases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93357166-04DD-4640-9F63-D97FAF308522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC4026E9-0CAD-4E8F-BEA6-E55EC15729F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4815" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision Histoy" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="107">
   <si>
     <t>S.No.</t>
   </si>
@@ -336,6 +336,18 @@
   </si>
   <si>
     <t>Genesis (The Beginning)</t>
+  </si>
+  <si>
+    <t>linker initial commit</t>
+  </si>
+  <si>
+    <t>initial linker commited</t>
+  </si>
+  <si>
+    <t>debug scipts updated</t>
+  </si>
+  <si>
+    <t>swd flashing and debugging working now</t>
   </si>
 </sst>
 </file>
@@ -558,7 +570,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -630,17 +642,18 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -942,107 +955,107 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="G3" s="73" t="s">
+      <c r="G3" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="73" t="s">
+      <c r="H3" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="I3" s="73" t="s">
+      <c r="I3" s="71" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="4" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C4" s="71" t="s">
+      <c r="C4" s="69" t="s">
         <v>93</v>
       </c>
-      <c r="D4" s="69" t="s">
+      <c r="D4" s="67" t="s">
         <v>102</v>
       </c>
-      <c r="G4" s="70">
+      <c r="G4" s="68">
         <v>45702</v>
       </c>
-      <c r="H4" s="69" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="69" t="s">
+      <c r="H4" s="67" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="67" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C5" s="71" t="s">
+      <c r="C5" s="69" t="s">
         <v>94</v>
       </c>
-      <c r="D5" s="69" t="s">
+      <c r="D5" s="67" t="s">
         <v>95</v>
       </c>
-      <c r="G5" s="69"/>
-      <c r="H5" s="69"/>
-      <c r="I5" s="69"/>
+      <c r="G5" s="67"/>
+      <c r="H5" s="67"/>
+      <c r="I5" s="67"/>
     </row>
     <row r="6" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C6" s="71" t="s">
+      <c r="C6" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="69" t="s">
+      <c r="D6" s="67" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="69"/>
-      <c r="H6" s="69"/>
-      <c r="I6" s="69"/>
+      <c r="G6" s="67"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="67"/>
     </row>
     <row r="7" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C7" s="71" t="s">
+      <c r="C7" s="69" t="s">
         <v>99</v>
       </c>
-      <c r="D7" s="69" t="s">
+      <c r="D7" s="67" t="s">
         <v>100</v>
       </c>
-      <c r="G7" s="69"/>
-      <c r="H7" s="69"/>
-      <c r="I7" s="69"/>
+      <c r="G7" s="67"/>
+      <c r="H7" s="67"/>
+      <c r="I7" s="67"/>
     </row>
     <row r="8" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C8" s="71" t="s">
+      <c r="C8" s="69" t="s">
         <v>101</v>
       </c>
-      <c r="D8" s="69" t="s">
+      <c r="D8" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="G8" s="69"/>
-      <c r="H8" s="69"/>
-      <c r="I8" s="69"/>
+      <c r="G8" s="67"/>
+      <c r="H8" s="67"/>
+      <c r="I8" s="67"/>
     </row>
     <row r="9" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C9" s="71"/>
-      <c r="D9" s="69"/>
-      <c r="G9" s="69"/>
-      <c r="H9" s="69"/>
-      <c r="I9" s="69"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="67"/>
+      <c r="G9" s="67"/>
+      <c r="H9" s="67"/>
+      <c r="I9" s="67"/>
     </row>
     <row r="10" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C10" s="71"/>
-      <c r="D10" s="69"/>
-      <c r="G10" s="69"/>
-      <c r="H10" s="69"/>
-      <c r="I10" s="69"/>
+      <c r="C10" s="69"/>
+      <c r="D10" s="67"/>
+      <c r="G10" s="67"/>
+      <c r="H10" s="67"/>
+      <c r="I10" s="67"/>
     </row>
     <row r="11" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C11" s="71"/>
-      <c r="D11" s="69"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="69"/>
-      <c r="I11" s="69"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="67"/>
+      <c r="G11" s="67"/>
+      <c r="H11" s="67"/>
+      <c r="I11" s="67"/>
     </row>
     <row r="12" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C12" s="71"/>
-      <c r="D12" s="69"/>
-      <c r="G12" s="69"/>
-      <c r="H12" s="69"/>
-      <c r="I12" s="69"/>
+      <c r="C12" s="69"/>
+      <c r="D12" s="67"/>
+      <c r="G12" s="67"/>
+      <c r="H12" s="67"/>
+      <c r="I12" s="67"/>
     </row>
     <row r="13" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C13" s="72"/>
+      <c r="C13" s="70"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1409,27 +1422,69 @@
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>13</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17" s="2">
+        <v>46145</v>
+      </c>
+      <c r="E17" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" t="s">
+        <v>7</v>
+      </c>
+      <c r="G17" t="s">
+        <v>7</v>
+      </c>
       <c r="L17" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="18" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>14</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D18" s="74">
+        <v>46159</v>
+      </c>
+      <c r="E18" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" t="s">
+        <v>7</v>
+      </c>
       <c r="L18" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="19" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="L19" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="L20" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="L21" t="s">
         <v>92</v>
       </c>
@@ -1518,10 +1573,10 @@
       <c r="I7" s="27"/>
       <c r="J7" s="27"/>
       <c r="K7" s="27"/>
-      <c r="L7" s="67" t="s">
+      <c r="L7" s="72" t="s">
         <v>43</v>
       </c>
-      <c r="M7" s="67"/>
+      <c r="M7" s="72"/>
       <c r="N7" s="27"/>
       <c r="O7" s="27"/>
       <c r="P7" s="27"/>
@@ -1698,10 +1753,10 @@
       <c r="I15" s="49"/>
       <c r="J15" s="49"/>
       <c r="K15" s="49"/>
-      <c r="L15" s="68" t="s">
+      <c r="L15" s="73" t="s">
         <v>61</v>
       </c>
-      <c r="M15" s="68"/>
+      <c r="M15" s="73"/>
       <c r="N15" s="49"/>
       <c r="O15" s="49"/>
       <c r="P15" s="49"/>

</xml_diff>

<commit_message>
linker and nvm plan update
</commit_message>
<xml_diff>
--- a/assets/Releases/Release_plan.xlsx
+++ b/assets/Releases/Release_plan.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\friday\rtos_pico\may17\Robo_dev\assets\Releases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E732EB72-A557-46B2-A852-9BF06534CC25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0347F8F2-B82E-4BA2-815A-0BDAB1170C40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4815" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-4815" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision Histoy" sheetId="1" r:id="rId1"/>
     <sheet name="Release" sheetId="2" r:id="rId2"/>
     <sheet name="HLD" sheetId="3" r:id="rId3"/>
+    <sheet name="backlogs" sheetId="6" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="120">
   <si>
     <t>S.No.</t>
   </si>
@@ -354,13 +355,46 @@
   </si>
   <si>
     <t>conan integration and build sh updated</t>
+  </si>
+  <si>
+    <t>S.no</t>
+  </si>
+  <si>
+    <t>backlogs</t>
+  </si>
+  <si>
+    <t>Linker</t>
+  </si>
+  <si>
+    <t>pegasus_origin</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1otueajQxHN-QnHXt9K9kVpu3_wXamMji/edit?usp=sharing&amp;ouid=108790899073558423476&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1NFU510WXUPIaXAXilT9mZKdLcdPsTjMy/edit?usp=sharing&amp;ouid=108790899073558423476&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1D_zF2kUfpSDvsSf33ci0dItezJaZXoTI/edit?usp=sharing&amp;ouid=108790899073558423476&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Current status</t>
+  </si>
+  <si>
+    <t>completion percentage</t>
+  </si>
+  <si>
+    <t>Not started</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -384,6 +418,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -573,10 +615,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -654,15 +697,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1272,7 +1319,7 @@
       <c r="L10" t="s">
         <v>81</v>
       </c>
-      <c r="M10" s="75">
+      <c r="M10" s="73">
         <v>0.3</v>
       </c>
     </row>
@@ -1509,7 +1556,7 @@
       <c r="L19" t="s">
         <v>90</v>
       </c>
-      <c r="M19" s="75">
+      <c r="M19" s="73">
         <v>0.5</v>
       </c>
     </row>
@@ -1607,10 +1654,10 @@
       <c r="I7" s="27"/>
       <c r="J7" s="27"/>
       <c r="K7" s="27"/>
-      <c r="L7" s="73" t="s">
+      <c r="L7" s="74" t="s">
         <v>43</v>
       </c>
-      <c r="M7" s="73"/>
+      <c r="M7" s="74"/>
       <c r="N7" s="27"/>
       <c r="O7" s="27"/>
       <c r="P7" s="27"/>
@@ -1787,10 +1834,10 @@
       <c r="I15" s="49"/>
       <c r="J15" s="49"/>
       <c r="K15" s="49"/>
-      <c r="L15" s="74" t="s">
+      <c r="L15" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="M15" s="74"/>
+      <c r="M15" s="75"/>
       <c r="N15" s="49"/>
       <c r="O15" s="49"/>
       <c r="P15" s="49"/>
@@ -1866,4 +1913,93 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03301342-AC1F-4EDE-8545-C68305A179F4}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="93.85546875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="76" t="s">
+        <v>115</v>
+      </c>
+      <c r="D2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E2" s="73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="76" t="s">
+        <v>114</v>
+      </c>
+      <c r="D3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E3" s="73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4" s="76" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E4" s="73">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" xr:uid="{92016FDA-4FB0-4370-995E-F5E2F8752AF0}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{FEA55184-503E-4E7D-A443-7C48351C9F45}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{1540347B-5624-4C50-9258-FF7B5FC3B0F7}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>